<commit_message>
added exterior variables. Addedd unit testing. Meteorite not included yet
</commit_message>
<xml_diff>
--- a/Documentation/cdcm_habitatmodel.xlsx
+++ b/Documentation/cdcm_habitatmodel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rashijainx/Documents/GitHub/cdcm_habitatmodel/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E5EFDB4-9F00-5540-B526-618DC722E535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4E1572-A017-644A-8354-47E4FDE4F884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="4" xr2:uid="{B9866D00-B1EC-D94E-AC1D-0DAFFC8F48F5}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{B9866D00-B1EC-D94E-AC1D-0DAFFC8F48F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements " sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="155">
   <si>
     <t xml:space="preserve">Node </t>
   </si>
@@ -525,6 +525,48 @@
   </si>
   <si>
     <t xml:space="preserve">Plan on next steps for modeling </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allows a Battery to Charge or Discharge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solar Arrays </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generates Charge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuclear Reactor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wiring </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carries Charge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voltage Regulator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regulates Charge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directs Charge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct Current Switching Unit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switches Charge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remote Powered Controller Module </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main Bus Switching Unit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provides Connectivity between Power Channel nad Multiple Downstream Loads </t>
   </si>
 </sst>
 </file>
@@ -1603,13 +1645,13 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.5" customWidth="1"/>
+    <col min="1" max="1" width="26.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="70.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1648,6 +1690,70 @@
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>